<commit_message>
updated ATTAINS Parameter across all criteria table
update R8 criteria tables to ensure all non-allowable ATTAINS parameter name are now allowable ones from ATTAINS from Hannah feedback.
</commit_message>
<xml_diff>
--- a/inst/extdata/blackfeet_tribe_criteria_crosswalk.xlsx
+++ b/inst/extdata/blackfeet_tribe_criteria_crosswalk.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kwong01\TADACommunityHub\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE2C29A-85A3-47DA-AE79-CECEF22B8E08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84252655-2FDA-46BC-8634-C1BD3E628908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28690" yWindow="-110" windowWidth="20710" windowHeight="11020" xr2:uid="{9CAA114B-CC1B-4AA7-94E1-A6CD4C5CB112}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9CAA114B-CC1B-4AA7-94E1-A6CD4C5CB112}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -302,9 +302,6 @@
     <t>Human Health - Organism</t>
   </si>
   <si>
-    <t>Mercury Methylmercury</t>
-  </si>
-  <si>
     <t>DIMETHYLMERCURY</t>
   </si>
   <si>
@@ -314,9 +311,6 @@
     <t>METHYLMERCURY(1+)</t>
   </si>
   <si>
-    <t>Chromium VI</t>
-  </si>
-  <si>
     <t>CHROMIUM(VI)</t>
   </si>
   <si>
@@ -368,9 +362,6 @@
     <t>e^(0.7409*ln(hardness)-4.719)*(1.101672-[ln(hardness)(0.041838)])</t>
   </si>
   <si>
-    <t>Chromium III</t>
-  </si>
-  <si>
     <t>CHROMIUM(III)</t>
   </si>
   <si>
@@ -431,9 +422,6 @@
     <t>IRON</t>
   </si>
   <si>
-    <t>Nitrates</t>
-  </si>
-  <si>
     <t>NITRATE</t>
   </si>
   <si>
@@ -449,15 +437,9 @@
     <t>arithmetic extremes</t>
   </si>
   <si>
-    <t>Solids Dissolved</t>
-  </si>
-  <si>
     <t>TOTAL DISSOLVED SOLIDS</t>
   </si>
   <si>
-    <t>E. coli</t>
-  </si>
-  <si>
     <t>Primary Recreation</t>
   </si>
   <si>
@@ -473,16 +455,10 @@
     <t>Percentile</t>
   </si>
   <si>
-    <t>Microcystin</t>
-  </si>
-  <si>
     <t>MICROCYSTIN</t>
   </si>
   <si>
     <t>n-samples in 3 10-day periods</t>
-  </si>
-  <si>
-    <t>Oxygen</t>
   </si>
   <si>
     <t>DISSOLVED OXYGEN (DO)</t>
@@ -1092,12 +1068,36 @@
   <si>
     <t>0.8876*(((0.0278/(1+10^(7.688-pH)))+(1.1994/(1+10^(pH-7.688))))*(2.126*10^(0.028*(20-max(Temperature,7)))))</t>
   </si>
+  <si>
+    <t>Methylmercury</t>
+  </si>
+  <si>
+    <t>CHROMIUM, HEXAVALENT</t>
+  </si>
+  <si>
+    <t>CHROMIUM, TRIVALENT, TOTAL</t>
+  </si>
+  <si>
+    <t>Nitrate</t>
+  </si>
+  <si>
+    <t>TOTAL DISSOLVED SOLIDS (TDS)</t>
+  </si>
+  <si>
+    <t>ESCHERICHIA COLI (E. COLI)</t>
+  </si>
+  <si>
+    <t>CYANOBACTERIA HEPATOTOXIC MICROCYSTINS</t>
+  </si>
+  <si>
+    <t>DISSOLVED OXYGEN</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1133,12 +1133,6 @@
       <name val="新細明體"/>
       <family val="2"/>
       <charset val="136"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1526,10 +1520,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{057945F5-944B-4C7F-AE65-F75344336C85}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AQ65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="19.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1664,7 +1658,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="5"/>
       <c r="B2" s="5" t="s">
         <v>43</v>
@@ -1733,7 +1727,7 @@
       <c r="AL2" s="5"/>
       <c r="AM2" s="5"/>
     </row>
-    <row r="3" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
         <v>43</v>
@@ -1804,7 +1798,7 @@
       <c r="AL3" s="5"/>
       <c r="AM3" s="5"/>
     </row>
-    <row r="4" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="5"/>
       <c r="B4" s="5" t="s">
         <v>43</v>
@@ -1875,7 +1869,7 @@
       <c r="AL4" s="5"/>
       <c r="AM4" s="5"/>
     </row>
-    <row r="5" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
       <c r="B5" s="5" t="s">
         <v>43</v>
@@ -1942,7 +1936,7 @@
       <c r="AL5" s="5"/>
       <c r="AM5" s="5"/>
     </row>
-    <row r="6" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="5"/>
       <c r="B6" s="5" t="s">
         <v>43</v>
@@ -2009,7 +2003,7 @@
       <c r="AL6" s="5"/>
       <c r="AM6" s="5"/>
     </row>
-    <row r="7" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="5"/>
       <c r="B7" s="5" t="s">
         <v>43</v>
@@ -2080,7 +2074,7 @@
       <c r="AL7" s="5"/>
       <c r="AM7" s="5"/>
     </row>
-    <row r="8" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="5"/>
       <c r="B8" s="5" t="s">
         <v>43</v>
@@ -2149,7 +2143,7 @@
       <c r="AL8" s="5"/>
       <c r="AM8" s="5"/>
     </row>
-    <row r="9" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="5"/>
       <c r="B9" s="5" t="s">
         <v>43</v>
@@ -2216,7 +2210,7 @@
       <c r="AL9" s="5"/>
       <c r="AM9" s="5"/>
     </row>
-    <row r="10" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A10" s="5"/>
       <c r="B10" s="5" t="s">
         <v>43</v>
@@ -2291,7 +2285,7 @@
       <c r="AL10" s="5"/>
       <c r="AM10" s="5"/>
     </row>
-    <row r="11" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="5"/>
       <c r="B11" s="5" t="s">
         <v>43</v>
@@ -2366,7 +2360,7 @@
       <c r="AL11" s="5"/>
       <c r="AM11" s="5"/>
     </row>
-    <row r="12" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
       <c r="B12" s="5" t="s">
         <v>43</v>
@@ -2435,7 +2429,7 @@
       <c r="AL12" s="5"/>
       <c r="AM12" s="5"/>
     </row>
-    <row r="13" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="5"/>
       <c r="B13" s="5" t="s">
         <v>43</v>
@@ -2506,7 +2500,7 @@
       <c r="AL13" s="5"/>
       <c r="AM13" s="5"/>
     </row>
-    <row r="14" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="5"/>
       <c r="B14" s="5" t="s">
         <v>43</v>
@@ -2577,7 +2571,7 @@
       <c r="AL14" s="5"/>
       <c r="AM14" s="5"/>
     </row>
-    <row r="15" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="B15" s="5" t="s">
         <v>43</v>
@@ -2646,7 +2640,7 @@
       <c r="AL15" s="5"/>
       <c r="AM15" s="5"/>
     </row>
-    <row r="16" spans="1:43" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" s="5"/>
       <c r="B16" s="5" t="s">
         <v>43</v>
@@ -2715,19 +2709,19 @@
       <c r="AL16" s="5"/>
       <c r="AM16" s="5"/>
     </row>
-    <row r="17" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
       <c r="B17" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>81</v>
+        <v>147</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>80</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
@@ -2746,7 +2740,7 @@
         <v>0.3</v>
       </c>
       <c r="P17" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="Q17" s="5">
         <v>30</v>
@@ -2782,19 +2776,19 @@
       <c r="AL17" s="5"/>
       <c r="AM17" s="5"/>
     </row>
-    <row r="18" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="5"/>
       <c r="B18" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>81</v>
+        <v>147</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>80</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
@@ -2813,7 +2807,7 @@
         <v>0.3</v>
       </c>
       <c r="P18" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="Q18" s="5">
         <v>30</v>
@@ -2849,19 +2843,19 @@
       <c r="AL18" s="5"/>
       <c r="AM18" s="5"/>
     </row>
-    <row r="19" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A19" s="5"/>
       <c r="B19" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>85</v>
+        <v>148</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>75</v>
@@ -2920,19 +2914,19 @@
       <c r="AL19" s="5"/>
       <c r="AM19" s="5"/>
     </row>
-    <row r="20" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>85</v>
+        <v>148</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F20" s="5" t="s">
         <v>75</v>
@@ -2991,19 +2985,19 @@
       <c r="AL20" s="5"/>
       <c r="AM20" s="5"/>
     </row>
-    <row r="21" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="5"/>
       <c r="B21" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>73</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>75</v>
@@ -3060,19 +3054,19 @@
       <c r="AL21" s="5"/>
       <c r="AM21" s="5"/>
     </row>
-    <row r="22" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A22" s="5"/>
       <c r="B22" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>80</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>75</v>
@@ -3129,7 +3123,7 @@
       <c r="AL22" s="5"/>
       <c r="AM22" s="5"/>
     </row>
-    <row r="23" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
       <c r="B23" s="5" t="s">
         <v>43</v>
@@ -3198,7 +3192,7 @@
       <c r="AL23" s="5"/>
       <c r="AM23" s="5"/>
     </row>
-    <row r="24" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A24" s="5"/>
       <c r="B24" s="5" t="s">
         <v>43</v>
@@ -3267,19 +3261,19 @@
       <c r="AL24" s="5"/>
       <c r="AM24" s="5"/>
     </row>
-    <row r="25" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="5"/>
       <c r="B25" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>73</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F25" s="5" t="s">
         <v>75</v>
@@ -3336,19 +3330,19 @@
       <c r="AL25" s="5"/>
       <c r="AM25" s="5"/>
     </row>
-    <row r="26" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A26" s="5"/>
       <c r="B26" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>80</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>75</v>
@@ -3405,19 +3399,19 @@
       <c r="AL26" s="5"/>
       <c r="AM26" s="5"/>
     </row>
-    <row r="27" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
       <c r="B27" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>73</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F27" s="5" t="s">
         <v>75</v>
@@ -3474,19 +3468,19 @@
       <c r="AL27" s="5"/>
       <c r="AM27" s="5"/>
     </row>
-    <row r="28" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A28" s="5"/>
       <c r="B28" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>80</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F28" s="5" t="s">
         <v>75</v>
@@ -3543,19 +3537,19 @@
       <c r="AL28" s="5"/>
       <c r="AM28" s="5"/>
     </row>
-    <row r="29" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A29" s="5"/>
       <c r="B29" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
@@ -3612,19 +3606,19 @@
       <c r="AL29" s="5"/>
       <c r="AM29" s="5"/>
     </row>
-    <row r="30" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="5"/>
       <c r="B30" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
@@ -3681,19 +3675,19 @@
       <c r="AL30" s="5"/>
       <c r="AM30" s="5"/>
     </row>
-    <row r="31" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="5"/>
       <c r="B31" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>73</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
@@ -3748,19 +3742,19 @@
       <c r="AL31" s="5"/>
       <c r="AM31" s="5"/>
     </row>
-    <row r="32" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A32" s="5"/>
       <c r="B32" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>80</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
@@ -3815,19 +3809,19 @@
       <c r="AL32" s="5"/>
       <c r="AM32" s="5"/>
     </row>
-    <row r="33" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>73</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
@@ -3846,7 +3840,7 @@
         <v>7000000</v>
       </c>
       <c r="P33" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="Q33" s="5">
         <v>1</v>
@@ -3882,19 +3876,19 @@
       <c r="AL33" s="5"/>
       <c r="AM33" s="5"/>
     </row>
-    <row r="34" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A34" s="5"/>
       <c r="B34" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>75</v>
@@ -3942,13 +3936,13 @@
       <c r="AC34" s="5"/>
       <c r="AD34" s="5"/>
       <c r="AE34" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="AF34" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG34" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="AH34" s="5">
         <v>1.1366719999999999</v>
@@ -3967,19 +3961,19 @@
       </c>
       <c r="AM34" s="5"/>
     </row>
-    <row r="35" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A35" s="5"/>
       <c r="B35" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>75</v>
@@ -4027,13 +4021,13 @@
       <c r="AC35" s="5"/>
       <c r="AD35" s="5"/>
       <c r="AE35" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="AF35" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG35" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="AH35" s="5">
         <v>1.101672</v>
@@ -4052,19 +4046,19 @@
       </c>
       <c r="AM35" s="5"/>
     </row>
-    <row r="36" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="5"/>
       <c r="B36" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>103</v>
+        <v>149</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F36" s="5" t="s">
         <v>75</v>
@@ -4112,13 +4106,13 @@
       <c r="AC36" s="5"/>
       <c r="AD36" s="5"/>
       <c r="AE36" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="AF36" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG36" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="AH36" s="5"/>
       <c r="AI36" s="5"/>
@@ -4133,19 +4127,19 @@
       </c>
       <c r="AM36" s="5"/>
     </row>
-    <row r="37" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A37" s="5"/>
       <c r="B37" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>103</v>
+        <v>149</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F37" s="5" t="s">
         <v>75</v>
@@ -4193,13 +4187,13 @@
       <c r="AC37" s="5"/>
       <c r="AD37" s="5"/>
       <c r="AE37" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="AF37" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG37" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="AH37" s="5"/>
       <c r="AI37" s="5"/>
@@ -4214,7 +4208,7 @@
       </c>
       <c r="AM37" s="5"/>
     </row>
-    <row r="38" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A38" s="5"/>
       <c r="B38" s="5" t="s">
         <v>43</v>
@@ -4274,13 +4268,13 @@
       <c r="AC38" s="5"/>
       <c r="AD38" s="5"/>
       <c r="AE38" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="AF38" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG38" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="AH38" s="5">
         <v>1.4620299999999999</v>
@@ -4299,7 +4293,7 @@
       </c>
       <c r="AM38" s="5"/>
     </row>
-    <row r="39" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A39" s="5"/>
       <c r="B39" s="5" t="s">
         <v>43</v>
@@ -4359,13 +4353,13 @@
       <c r="AC39" s="5"/>
       <c r="AD39" s="5"/>
       <c r="AE39" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="AF39" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG39" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="AH39" s="5">
         <v>1.4620299999999999</v>
@@ -4384,19 +4378,19 @@
       </c>
       <c r="AM39" s="5"/>
     </row>
-    <row r="40" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A40" s="5"/>
       <c r="B40" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F40" s="5" t="s">
         <v>75</v>
@@ -4444,13 +4438,13 @@
       <c r="AC40" s="5"/>
       <c r="AD40" s="5"/>
       <c r="AE40" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="AF40" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG40" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="AH40" s="5"/>
       <c r="AI40" s="5"/>
@@ -4465,19 +4459,19 @@
       </c>
       <c r="AM40" s="5"/>
     </row>
-    <row r="41" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A41" s="5"/>
       <c r="B41" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F41" s="5" t="s">
         <v>75</v>
@@ -4525,13 +4519,13 @@
       <c r="AC41" s="5"/>
       <c r="AD41" s="5"/>
       <c r="AE41" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="AF41" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG41" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="AH41" s="5"/>
       <c r="AI41" s="5"/>
@@ -4546,19 +4540,19 @@
       </c>
       <c r="AM41" s="5"/>
     </row>
-    <row r="42" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A42" s="5"/>
       <c r="B42" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F42" s="5" t="s">
         <v>75</v>
@@ -4606,13 +4600,13 @@
       <c r="AC42" s="5"/>
       <c r="AD42" s="5"/>
       <c r="AE42" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="AF42" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG42" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="AH42" s="5"/>
       <c r="AI42" s="5"/>
@@ -4627,19 +4621,19 @@
       </c>
       <c r="AM42" s="5"/>
     </row>
-    <row r="43" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A43" s="5"/>
       <c r="B43" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F43" s="5" t="s">
         <v>75</v>
@@ -4687,13 +4681,13 @@
       <c r="AC43" s="5"/>
       <c r="AD43" s="5"/>
       <c r="AE43" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="AF43" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG43" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="AH43" s="5"/>
       <c r="AI43" s="5"/>
@@ -4708,19 +4702,19 @@
       </c>
       <c r="AM43" s="5"/>
     </row>
-    <row r="44" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A44" s="5"/>
       <c r="B44" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F44" s="5" t="s">
         <v>75</v>
@@ -4768,13 +4762,13 @@
       <c r="AC44" s="5"/>
       <c r="AD44" s="5"/>
       <c r="AE44" s="5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="AF44" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG44" s="5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="AH44" s="5"/>
       <c r="AI44" s="5"/>
@@ -4789,19 +4783,19 @@
       </c>
       <c r="AM44" s="5"/>
     </row>
-    <row r="45" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A45" s="5"/>
       <c r="B45" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>73</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
@@ -4856,19 +4850,19 @@
       <c r="AL45" s="5"/>
       <c r="AM45" s="5"/>
     </row>
-    <row r="46" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A46" s="5"/>
       <c r="B46" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
@@ -4925,19 +4919,19 @@
       <c r="AL46" s="5"/>
       <c r="AM46" s="5"/>
     </row>
-    <row r="47" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A47" s="5"/>
       <c r="B47" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
@@ -4994,19 +4988,19 @@
       <c r="AL47" s="5"/>
       <c r="AM47" s="5"/>
     </row>
-    <row r="48" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A48" s="5"/>
       <c r="B48" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F48" s="5" t="s">
         <v>56</v>
@@ -5065,19 +5059,19 @@
       <c r="AL48" s="5"/>
       <c r="AM48" s="5"/>
     </row>
-    <row r="49" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A49" s="5"/>
       <c r="B49" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F49" s="5" t="s">
         <v>56</v>
@@ -5136,19 +5130,19 @@
       <c r="AL49" s="5"/>
       <c r="AM49" s="5"/>
     </row>
-    <row r="50" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="5"/>
       <c r="B50" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
@@ -5205,19 +5199,19 @@
       <c r="AL50" s="5"/>
       <c r="AM50" s="5"/>
     </row>
-    <row r="51" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A51" s="5"/>
       <c r="B51" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>73</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
@@ -5272,19 +5266,19 @@
       <c r="AL51" s="5"/>
       <c r="AM51" s="5"/>
     </row>
-    <row r="52" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A52" s="5"/>
       <c r="B52" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
@@ -5307,7 +5301,7 @@
         <v>9</v>
       </c>
       <c r="P52" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="Q52" s="5">
         <v>7</v>
@@ -5316,7 +5310,7 @@
         <v>51</v>
       </c>
       <c r="S52" s="5" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="T52" s="5">
         <v>1</v>
@@ -5343,19 +5337,19 @@
       <c r="AL52" s="5"/>
       <c r="AM52" s="5"/>
     </row>
-    <row r="53" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A53" s="5"/>
       <c r="B53" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>73</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
@@ -5376,7 +5370,7 @@
         <v>9</v>
       </c>
       <c r="P53" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="Q53" s="5">
         <v>1</v>
@@ -5385,7 +5379,7 @@
         <v>51</v>
       </c>
       <c r="S53" s="5" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="T53" s="5">
         <v>1</v>
@@ -5412,19 +5406,19 @@
       <c r="AL53" s="5"/>
       <c r="AM53" s="5"/>
     </row>
-    <row r="54" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A54" s="5"/>
       <c r="B54" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>73</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="F54" s="5" t="s">
         <v>56</v>
@@ -5481,19 +5475,19 @@
       <c r="AL54" s="5"/>
       <c r="AM54" s="5"/>
     </row>
-    <row r="55" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A55" s="5"/>
       <c r="B55" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="F55" s="5"/>
       <c r="G55" s="5"/>
@@ -5512,7 +5506,7 @@
         <v>126</v>
       </c>
       <c r="P55" s="5" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="Q55" s="5">
         <v>90</v>
@@ -5521,7 +5515,7 @@
         <v>51</v>
       </c>
       <c r="S55" s="5" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="T55" s="5">
         <v>1</v>
@@ -5548,19 +5542,19 @@
       <c r="AL55" s="5"/>
       <c r="AM55" s="5"/>
     </row>
-    <row r="56" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A56" s="5"/>
       <c r="B56" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="F56" s="5"/>
       <c r="G56" s="5"/>
@@ -5579,7 +5573,7 @@
         <v>410</v>
       </c>
       <c r="P56" s="5" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="Q56" s="5">
         <v>90</v>
@@ -5594,7 +5588,7 @@
         <v>10</v>
       </c>
       <c r="U56" s="5" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="V56" s="5"/>
       <c r="W56" s="5"/>
@@ -5615,19 +5609,19 @@
       <c r="AL56" s="5"/>
       <c r="AM56" s="5"/>
     </row>
-    <row r="57" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A57" s="5"/>
       <c r="B57" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F57" s="5"/>
       <c r="G57" s="5"/>
@@ -5661,7 +5655,7 @@
         <v>1</v>
       </c>
       <c r="U57" s="5" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="V57" s="5"/>
       <c r="W57" s="5"/>
@@ -5682,19 +5676,19 @@
       <c r="AL57" s="5"/>
       <c r="AM57" s="5"/>
     </row>
-    <row r="58" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A58" s="5"/>
       <c r="B58" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F58" s="5"/>
       <c r="G58" s="5"/>
@@ -5728,7 +5722,7 @@
         <v>1</v>
       </c>
       <c r="U58" s="5" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="V58" s="5"/>
       <c r="W58" s="5"/>
@@ -5749,22 +5743,22 @@
       <c r="AL58" s="5"/>
       <c r="AM58" s="5"/>
     </row>
-    <row r="59" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A59" s="5"/>
       <c r="B59" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="G59" s="5"/>
       <c r="H59" s="5"/>
@@ -5774,7 +5768,7 @@
       </c>
       <c r="K59" s="5"/>
       <c r="L59" s="5" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="M59" s="5" t="s">
         <v>49</v>
@@ -5784,7 +5778,7 @@
       </c>
       <c r="O59" s="5"/>
       <c r="P59" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="Q59" s="5">
         <v>7</v>
@@ -5820,22 +5814,22 @@
       <c r="AL59" s="5"/>
       <c r="AM59" s="5"/>
     </row>
-    <row r="60" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A60" s="5"/>
       <c r="B60" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="G60" s="5"/>
       <c r="H60" s="5"/>
@@ -5845,7 +5839,7 @@
       </c>
       <c r="K60" s="5"/>
       <c r="L60" s="5" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="M60" s="5" t="s">
         <v>49</v>
@@ -5855,7 +5849,7 @@
       </c>
       <c r="O60" s="5"/>
       <c r="P60" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="Q60" s="5">
         <v>30</v>
@@ -5897,16 +5891,16 @@
         <v>43</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="G61" s="5"/>
       <c r="H61" s="5"/>
@@ -5916,7 +5910,7 @@
       </c>
       <c r="K61" s="5"/>
       <c r="L61" s="5" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="M61" s="5" t="s">
         <v>49</v>
@@ -5926,7 +5920,7 @@
       </c>
       <c r="O61" s="5"/>
       <c r="P61" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="Q61" s="5">
         <v>7</v>
@@ -5935,7 +5929,7 @@
         <v>51</v>
       </c>
       <c r="S61" s="5" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="T61" s="5">
         <v>1</v>
@@ -5962,22 +5956,22 @@
       <c r="AL61" s="5"/>
       <c r="AM61" s="5"/>
     </row>
-    <row r="62" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A62" s="5"/>
       <c r="B62" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="G62" s="5"/>
       <c r="H62" s="5"/>
@@ -5987,7 +5981,7 @@
       </c>
       <c r="K62" s="5"/>
       <c r="L62" s="5" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="M62" s="5" t="s">
         <v>49</v>
@@ -5997,7 +5991,7 @@
       </c>
       <c r="O62" s="5"/>
       <c r="P62" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="Q62" s="5">
         <v>1</v>
@@ -6006,7 +6000,7 @@
         <v>51</v>
       </c>
       <c r="S62" s="5" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="T62" s="5">
         <v>1</v>
@@ -6033,22 +6027,22 @@
       <c r="AL62" s="5"/>
       <c r="AM62" s="5"/>
     </row>
-    <row r="63" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A63" s="5"/>
       <c r="B63" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="G63" s="5"/>
       <c r="H63" s="5"/>
@@ -6058,7 +6052,7 @@
       </c>
       <c r="K63" s="5"/>
       <c r="L63" s="5" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="M63" s="5" t="s">
         <v>49</v>
@@ -6068,7 +6062,7 @@
       </c>
       <c r="O63" s="5"/>
       <c r="P63" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="Q63" s="5">
         <v>1</v>
@@ -6077,7 +6071,7 @@
         <v>51</v>
       </c>
       <c r="S63" s="5" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="T63" s="5">
         <v>1</v>
@@ -6104,19 +6098,19 @@
       <c r="AL63" s="5"/>
       <c r="AM63" s="5"/>
     </row>
-    <row r="64" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A64" s="5"/>
       <c r="B64" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="F64" s="5" t="s">
         <v>56</v>
@@ -6137,7 +6131,7 @@
       <c r="N64" s="5"/>
       <c r="O64" s="5"/>
       <c r="P64" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="Q64" s="5">
         <v>1</v>
@@ -6164,13 +6158,13 @@
       <c r="AC64" s="5"/>
       <c r="AD64" s="5"/>
       <c r="AE64" s="5" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="AF64" s="5" t="s">
         <v>71</v>
       </c>
       <c r="AG64" s="5" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="AH64" s="5"/>
       <c r="AI64" s="5"/>
@@ -6179,19 +6173,19 @@
       <c r="AL64" s="5"/>
       <c r="AM64" s="5"/>
     </row>
-    <row r="65" spans="1:39" s="4" customFormat="1" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A65" s="5"/>
       <c r="B65" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="F65" s="5" t="s">
         <v>56</v>
@@ -6212,7 +6206,7 @@
       <c r="N65" s="5"/>
       <c r="O65" s="5"/>
       <c r="P65" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="Q65" s="5">
         <v>30</v>
@@ -6239,13 +6233,13 @@
       <c r="AC65" s="5"/>
       <c r="AD65" s="5"/>
       <c r="AE65" s="5" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="AF65" s="5" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="AG65" s="5" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="AH65" s="5"/>
       <c r="AI65" s="5"/>
@@ -6255,13 +6249,7 @@
       <c r="AM65" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AQ65" xr:uid="{057945F5-944B-4C7F-AE65-F75344336C85}">
-    <filterColumn colId="18">
-      <filters>
-        <filter val="arithmetic mean min"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:AQ65" xr:uid="{057945F5-944B-4C7F-AE65-F75344336C85}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
update e.coli magnitude units to CFU/100ML
changed from #/100mL to CFU/100ML.
</commit_message>
<xml_diff>
--- a/inst/extdata/blackfeet_tribe_criteria_crosswalk.xlsx
+++ b/inst/extdata/blackfeet_tribe_criteria_crosswalk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tetratechinc-my.sharepoint.com/personal/sheila_saia_tetratech_com/Documents/Documents/github/TADACommunityHub/inst/extdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kwong01\TADACommunityHub\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:1_{82E9182B-18E3-4224-BFD1-BB785E56107E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E74FD0B-30E2-414D-9D8E-FB136CACD6F8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB60F2B-4287-4E1F-B327-A1104AEB08CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9CAA114B-CC1B-4AA7-94E1-A6CD4C5CB112}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9CAA114B-CC1B-4AA7-94E1-A6CD4C5CB112}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -383,9 +383,6 @@
     <t>ESCHERICHIA COLI</t>
   </si>
   <si>
-    <t>#/100mL</t>
-  </si>
-  <si>
     <t>geometric mean</t>
   </si>
   <si>
@@ -498,6 +495,9 @@
   </si>
   <si>
     <t>0.986*e^(0.8473*ln(hardness)+0.884)</t>
+  </si>
+  <si>
+    <t>CFU/100ML</t>
   </si>
 </sst>
 </file>
@@ -907,19 +907,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{057945F5-944B-4C7F-AE65-F75344336C85}">
   <dimension ref="A1:AP65"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="9.140625" style="3"/>
+    <col min="1" max="2" width="9.1796875" style="3"/>
     <col min="3" max="3" width="27" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="18" width="9.140625" style="3"/>
-    <col min="19" max="19" width="19.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="31" width="9.140625" style="3"/>
-    <col min="32" max="32" width="12.42578125" style="3" customWidth="1"/>
-    <col min="33" max="16384" width="9.140625" style="3"/>
+    <col min="4" max="4" width="31.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="18" width="9.1796875" style="3"/>
+    <col min="19" max="19" width="19.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="31" width="9.1796875" style="3"/>
+    <col min="32" max="32" width="12.453125" style="3" customWidth="1"/>
+    <col min="33" max="16384" width="9.1796875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:42" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1047,7 +1047,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="4"/>
       <c r="B2" s="4" t="s">
         <v>42</v>
@@ -1119,7 +1119,7 @@
       <c r="AO2" s="6"/>
       <c r="AP2" s="6"/>
     </row>
-    <row r="3" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
         <v>42</v>
@@ -1193,7 +1193,7 @@
       <c r="AO3" s="6"/>
       <c r="AP3" s="6"/>
     </row>
-    <row r="4" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
         <v>42</v>
@@ -1267,7 +1267,7 @@
       <c r="AO4" s="6"/>
       <c r="AP4" s="6"/>
     </row>
-    <row r="5" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
         <v>42</v>
@@ -1337,7 +1337,7 @@
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
     </row>
-    <row r="6" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4"/>
       <c r="B6" s="4" t="s">
         <v>42</v>
@@ -1407,7 +1407,7 @@
       <c r="AO6" s="6"/>
       <c r="AP6" s="6"/>
     </row>
-    <row r="7" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4"/>
       <c r="B7" s="4" t="s">
         <v>42</v>
@@ -1481,7 +1481,7 @@
       <c r="AO7" s="6"/>
       <c r="AP7" s="6"/>
     </row>
-    <row r="8" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
         <v>42</v>
@@ -1553,7 +1553,7 @@
       <c r="AO8" s="6"/>
       <c r="AP8" s="6"/>
     </row>
-    <row r="9" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="4"/>
       <c r="B9" s="4" t="s">
         <v>42</v>
@@ -1623,7 +1623,7 @@
       <c r="AO9" s="6"/>
       <c r="AP9" s="6"/>
     </row>
-    <row r="10" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
       <c r="B10" s="4" t="s">
         <v>42</v>
@@ -1699,7 +1699,7 @@
       <c r="AO10" s="6"/>
       <c r="AP10" s="6"/>
     </row>
-    <row r="11" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="4" t="s">
         <v>42</v>
@@ -1775,7 +1775,7 @@
       <c r="AO11" s="6"/>
       <c r="AP11" s="6"/>
     </row>
-    <row r="12" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
       <c r="B12" s="4" t="s">
         <v>42</v>
@@ -1784,7 +1784,7 @@
         <v>71</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>72</v>
@@ -1847,7 +1847,7 @@
       <c r="AO12" s="6"/>
       <c r="AP12" s="6"/>
     </row>
-    <row r="13" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
       <c r="B13" s="4" t="s">
         <v>42</v>
@@ -1921,7 +1921,7 @@
       <c r="AO13" s="6"/>
       <c r="AP13" s="6"/>
     </row>
-    <row r="14" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
         <v>42</v>
@@ -1995,7 +1995,7 @@
       <c r="AO14" s="6"/>
       <c r="AP14" s="6"/>
     </row>
-    <row r="15" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="4"/>
       <c r="B15" s="4" t="s">
         <v>42</v>
@@ -2004,7 +2004,7 @@
         <v>76</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>77</v>
@@ -2067,7 +2067,7 @@
       <c r="AO15" s="6"/>
       <c r="AP15" s="6"/>
     </row>
-    <row r="16" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" s="4"/>
       <c r="B16" s="4" t="s">
         <v>42</v>
@@ -2139,13 +2139,13 @@
       <c r="AO16" s="6"/>
       <c r="AP16" s="6"/>
     </row>
-    <row r="17" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" s="4"/>
       <c r="B17" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>44</v>
@@ -2209,13 +2209,13 @@
       <c r="AO17" s="6"/>
       <c r="AP17" s="6"/>
     </row>
-    <row r="18" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="4"/>
       <c r="B18" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>44</v>
@@ -2279,13 +2279,13 @@
       <c r="AO18" s="6"/>
       <c r="AP18" s="6"/>
     </row>
-    <row r="19" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A19" s="4"/>
       <c r="B19" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>44</v>
@@ -2353,13 +2353,13 @@
       <c r="AO19" s="6"/>
       <c r="AP19" s="6"/>
     </row>
-    <row r="20" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A20" s="4"/>
       <c r="B20" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>44</v>
@@ -2427,7 +2427,7 @@
       <c r="AO20" s="6"/>
       <c r="AP20" s="6"/>
     </row>
-    <row r="21" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="4"/>
       <c r="B21" s="4" t="s">
         <v>42</v>
@@ -2436,7 +2436,7 @@
         <v>82</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>83</v>
@@ -2499,7 +2499,7 @@
       <c r="AO21" s="6"/>
       <c r="AP21" s="6"/>
     </row>
-    <row r="22" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A22" s="4"/>
       <c r="B22" s="4" t="s">
         <v>42</v>
@@ -2571,7 +2571,7 @@
       <c r="AO22" s="6"/>
       <c r="AP22" s="6"/>
     </row>
-    <row r="23" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A23" s="4"/>
       <c r="B23" s="4" t="s">
         <v>42</v>
@@ -2580,7 +2580,7 @@
         <v>53</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>54</v>
@@ -2643,7 +2643,7 @@
       <c r="AO23" s="6"/>
       <c r="AP23" s="6"/>
     </row>
-    <row r="24" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A24" s="4"/>
       <c r="B24" s="4" t="s">
         <v>42</v>
@@ -2715,7 +2715,7 @@
       <c r="AO24" s="6"/>
       <c r="AP24" s="6"/>
     </row>
-    <row r="25" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="4"/>
       <c r="B25" s="4" t="s">
         <v>42</v>
@@ -2724,7 +2724,7 @@
         <v>84</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>85</v>
@@ -2787,7 +2787,7 @@
       <c r="AO25" s="6"/>
       <c r="AP25" s="6"/>
     </row>
-    <row r="26" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A26" s="4"/>
       <c r="B26" s="4" t="s">
         <v>42</v>
@@ -2859,7 +2859,7 @@
       <c r="AO26" s="6"/>
       <c r="AP26" s="6"/>
     </row>
-    <row r="27" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
         <v>42</v>
@@ -2868,7 +2868,7 @@
         <v>86</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>87</v>
@@ -2931,7 +2931,7 @@
       <c r="AO27" s="6"/>
       <c r="AP27" s="6"/>
     </row>
-    <row r="28" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A28" s="4"/>
       <c r="B28" s="4" t="s">
         <v>42</v>
@@ -3003,7 +3003,7 @@
       <c r="AO28" s="6"/>
       <c r="AP28" s="6"/>
     </row>
-    <row r="29" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A29" s="4"/>
       <c r="B29" s="4" t="s">
         <v>42</v>
@@ -3075,7 +3075,7 @@
       <c r="AO29" s="6"/>
       <c r="AP29" s="6"/>
     </row>
-    <row r="30" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="4"/>
       <c r="B30" s="4" t="s">
         <v>42</v>
@@ -3147,7 +3147,7 @@
       <c r="AO30" s="6"/>
       <c r="AP30" s="6"/>
     </row>
-    <row r="31" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="4"/>
       <c r="B31" s="4" t="s">
         <v>42</v>
@@ -3156,7 +3156,7 @@
         <v>88</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>89</v>
@@ -3217,7 +3217,7 @@
       <c r="AO31" s="6"/>
       <c r="AP31" s="6"/>
     </row>
-    <row r="32" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A32" s="4"/>
       <c r="B32" s="4" t="s">
         <v>42</v>
@@ -3287,7 +3287,7 @@
       <c r="AO32" s="6"/>
       <c r="AP32" s="6"/>
     </row>
-    <row r="33" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A33" s="4"/>
       <c r="B33" s="4" t="s">
         <v>42</v>
@@ -3296,7 +3296,7 @@
         <v>90</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>91</v>
@@ -3357,7 +3357,7 @@
       <c r="AO33" s="6"/>
       <c r="AP33" s="6"/>
     </row>
-    <row r="34" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A34" s="4"/>
       <c r="B34" s="4" t="s">
         <v>42</v>
@@ -3420,7 +3420,7 @@
         <v>95</v>
       </c>
       <c r="AF34" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AG34" s="4">
         <v>1.1366719999999999</v>
@@ -3443,7 +3443,7 @@
       <c r="AO34" s="6"/>
       <c r="AP34" s="6"/>
     </row>
-    <row r="35" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A35" s="4"/>
       <c r="B35" s="4" t="s">
         <v>42</v>
@@ -3506,7 +3506,7 @@
         <v>95</v>
       </c>
       <c r="AF35" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AG35" s="4">
         <v>1.101672</v>
@@ -3529,13 +3529,13 @@
       <c r="AO35" s="6"/>
       <c r="AP35" s="6"/>
     </row>
-    <row r="36" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="4"/>
       <c r="B36" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>44</v>
@@ -3592,7 +3592,7 @@
         <v>95</v>
       </c>
       <c r="AF36" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AG36" s="4"/>
       <c r="AH36" s="4"/>
@@ -3611,13 +3611,13 @@
       <c r="AO36" s="6"/>
       <c r="AP36" s="6"/>
     </row>
-    <row r="37" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A37" s="4"/>
       <c r="B37" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>44</v>
@@ -3674,7 +3674,7 @@
         <v>95</v>
       </c>
       <c r="AF37" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AG37" s="4"/>
       <c r="AH37" s="4"/>
@@ -3693,7 +3693,7 @@
       <c r="AO37" s="6"/>
       <c r="AP37" s="6"/>
     </row>
-    <row r="38" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A38" s="4"/>
       <c r="B38" s="4" t="s">
         <v>42</v>
@@ -3756,7 +3756,7 @@
         <v>95</v>
       </c>
       <c r="AF38" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AG38" s="4">
         <v>1.4620299999999999</v>
@@ -3779,7 +3779,7 @@
       <c r="AO38" s="6"/>
       <c r="AP38" s="6"/>
     </row>
-    <row r="39" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
         <v>42</v>
@@ -3842,7 +3842,7 @@
         <v>95</v>
       </c>
       <c r="AF39" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AG39" s="4">
         <v>1.4620299999999999</v>
@@ -3865,7 +3865,7 @@
       <c r="AO39" s="6"/>
       <c r="AP39" s="6"/>
     </row>
-    <row r="40" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
         <v>42</v>
@@ -3928,7 +3928,7 @@
         <v>95</v>
       </c>
       <c r="AF40" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AG40" s="4"/>
       <c r="AH40" s="4"/>
@@ -3947,7 +3947,7 @@
       <c r="AO40" s="6"/>
       <c r="AP40" s="6"/>
     </row>
-    <row r="41" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
         <v>42</v>
@@ -4010,7 +4010,7 @@
         <v>95</v>
       </c>
       <c r="AF41" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AG41" s="4"/>
       <c r="AH41" s="4"/>
@@ -4029,7 +4029,7 @@
       <c r="AO41" s="6"/>
       <c r="AP41" s="6"/>
     </row>
-    <row r="42" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A42" s="4"/>
       <c r="B42" s="4" t="s">
         <v>42</v>
@@ -4092,7 +4092,7 @@
         <v>95</v>
       </c>
       <c r="AF42" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AG42" s="4"/>
       <c r="AH42" s="4"/>
@@ -4111,7 +4111,7 @@
       <c r="AO42" s="6"/>
       <c r="AP42" s="6"/>
     </row>
-    <row r="43" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A43" s="4"/>
       <c r="B43" s="4" t="s">
         <v>42</v>
@@ -4174,7 +4174,7 @@
         <v>95</v>
       </c>
       <c r="AF43" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AG43" s="4"/>
       <c r="AH43" s="4"/>
@@ -4193,7 +4193,7 @@
       <c r="AO43" s="6"/>
       <c r="AP43" s="6"/>
     </row>
-    <row r="44" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A44" s="4"/>
       <c r="B44" s="4" t="s">
         <v>42</v>
@@ -4256,7 +4256,7 @@
         <v>95</v>
       </c>
       <c r="AF44" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AG44" s="4"/>
       <c r="AH44" s="4"/>
@@ -4275,7 +4275,7 @@
       <c r="AO44" s="6"/>
       <c r="AP44" s="6"/>
     </row>
-    <row r="45" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A45" s="4"/>
       <c r="B45" s="4" t="s">
         <v>42</v>
@@ -4284,7 +4284,7 @@
         <v>99</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>100</v>
@@ -4345,7 +4345,7 @@
       <c r="AO45" s="6"/>
       <c r="AP45" s="6"/>
     </row>
-    <row r="46" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A46" s="4"/>
       <c r="B46" s="4" t="s">
         <v>42</v>
@@ -4417,7 +4417,7 @@
       <c r="AO46" s="6"/>
       <c r="AP46" s="6"/>
     </row>
-    <row r="47" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A47" s="4"/>
       <c r="B47" s="4" t="s">
         <v>42</v>
@@ -4489,7 +4489,7 @@
       <c r="AO47" s="6"/>
       <c r="AP47" s="6"/>
     </row>
-    <row r="48" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A48" s="4"/>
       <c r="B48" s="4" t="s">
         <v>42</v>
@@ -4563,7 +4563,7 @@
       <c r="AO48" s="6"/>
       <c r="AP48" s="6"/>
     </row>
-    <row r="49" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A49" s="4"/>
       <c r="B49" s="4" t="s">
         <v>42</v>
@@ -4637,7 +4637,7 @@
       <c r="AO49" s="6"/>
       <c r="AP49" s="6"/>
     </row>
-    <row r="50" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="4"/>
       <c r="B50" s="4" t="s">
         <v>42</v>
@@ -4709,16 +4709,16 @@
       <c r="AO50" s="6"/>
       <c r="AP50" s="6"/>
     </row>
-    <row r="51" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A51" s="4"/>
       <c r="B51" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>107</v>
@@ -4779,7 +4779,7 @@
       <c r="AO51" s="6"/>
       <c r="AP51" s="6"/>
     </row>
-    <row r="52" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A52" s="4"/>
       <c r="B52" s="4" t="s">
         <v>42</v>
@@ -4853,7 +4853,7 @@
       <c r="AO52" s="6"/>
       <c r="AP52" s="6"/>
     </row>
-    <row r="53" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A53" s="4"/>
       <c r="B53" s="4" t="s">
         <v>42</v>
@@ -4862,7 +4862,7 @@
         <v>108</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E53" s="4" t="s">
         <v>109</v>
@@ -4925,16 +4925,16 @@
       <c r="AO53" s="6"/>
       <c r="AP53" s="6"/>
     </row>
-    <row r="54" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A54" s="4"/>
       <c r="B54" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E54" s="4" t="s">
         <v>112</v>
@@ -4997,16 +4997,16 @@
       <c r="AO54" s="6"/>
       <c r="AP54" s="6"/>
     </row>
-    <row r="55" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A55" s="4"/>
       <c r="B55" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E55" s="4" t="s">
         <v>113</v>
@@ -5028,7 +5028,7 @@
         <v>126</v>
       </c>
       <c r="P55" s="4" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="Q55" s="4">
         <v>90</v>
@@ -5037,7 +5037,7 @@
         <v>50</v>
       </c>
       <c r="S55" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="T55" s="4">
         <v>1</v>
@@ -5067,16 +5067,16 @@
       <c r="AO55" s="6"/>
       <c r="AP55" s="6"/>
     </row>
-    <row r="56" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A56" s="4"/>
       <c r="B56" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E56" s="4" t="s">
         <v>113</v>
@@ -5098,7 +5098,7 @@
         <v>410</v>
       </c>
       <c r="P56" s="4" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="Q56" s="4">
         <v>90</v>
@@ -5113,7 +5113,7 @@
         <v>10</v>
       </c>
       <c r="U56" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="V56" s="4"/>
       <c r="W56" s="4"/>
@@ -5137,19 +5137,19 @@
       <c r="AO56" s="6"/>
       <c r="AP56" s="6"/>
     </row>
-    <row r="57" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A57" s="4"/>
       <c r="B57" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
@@ -5183,7 +5183,7 @@
         <v>1</v>
       </c>
       <c r="U57" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V57" s="4"/>
       <c r="W57" s="4"/>
@@ -5207,19 +5207,19 @@
       <c r="AO57" s="6"/>
       <c r="AP57" s="6"/>
     </row>
-    <row r="58" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A58" s="4"/>
       <c r="B58" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
@@ -5253,7 +5253,7 @@
         <v>1</v>
       </c>
       <c r="U58" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V58" s="4"/>
       <c r="W58" s="4"/>
@@ -5277,22 +5277,22 @@
       <c r="AO58" s="6"/>
       <c r="AP58" s="6"/>
     </row>
-    <row r="59" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A59" s="4"/>
       <c r="B59" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E59" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F59" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="F59" s="4" t="s">
-        <v>120</v>
       </c>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="K59" s="4"/>
       <c r="L59" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M59" s="4" t="s">
         <v>48</v>
@@ -5312,7 +5312,7 @@
       </c>
       <c r="O59" s="4"/>
       <c r="P59" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q59" s="4">
         <v>7</v>
@@ -5351,22 +5351,22 @@
       <c r="AO59" s="6"/>
       <c r="AP59" s="6"/>
     </row>
-    <row r="60" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A60" s="4"/>
       <c r="B60" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E60" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F60" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="F60" s="4" t="s">
-        <v>120</v>
       </c>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="K60" s="4"/>
       <c r="L60" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M60" s="4" t="s">
         <v>48</v>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="O60" s="4"/>
       <c r="P60" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q60" s="4">
         <v>30</v>
@@ -5425,22 +5425,22 @@
       <c r="AO60" s="6"/>
       <c r="AP60" s="6"/>
     </row>
-    <row r="61" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A61" s="4"/>
       <c r="B61" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E61" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F61" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="F61" s="4" t="s">
-        <v>120</v>
       </c>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -5450,7 +5450,7 @@
       </c>
       <c r="K61" s="4"/>
       <c r="L61" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M61" s="4" t="s">
         <v>48</v>
@@ -5460,7 +5460,7 @@
       </c>
       <c r="O61" s="4"/>
       <c r="P61" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q61" s="4">
         <v>7</v>
@@ -5469,7 +5469,7 @@
         <v>50</v>
       </c>
       <c r="S61" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="T61" s="4">
         <v>1</v>
@@ -5499,22 +5499,22 @@
       <c r="AO61" s="6"/>
       <c r="AP61" s="6"/>
     </row>
-    <row r="62" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A62" s="4"/>
       <c r="B62" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E62" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F62" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="F62" s="4" t="s">
-        <v>120</v>
       </c>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -5524,7 +5524,7 @@
       </c>
       <c r="K62" s="4"/>
       <c r="L62" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M62" s="4" t="s">
         <v>48</v>
@@ -5534,7 +5534,7 @@
       </c>
       <c r="O62" s="4"/>
       <c r="P62" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q62" s="4">
         <v>1</v>
@@ -5543,7 +5543,7 @@
         <v>50</v>
       </c>
       <c r="S62" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T62" s="4">
         <v>1</v>
@@ -5573,22 +5573,22 @@
       <c r="AO62" s="6"/>
       <c r="AP62" s="6"/>
     </row>
-    <row r="63" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A63" s="4"/>
       <c r="B63" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E63" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F63" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="F63" s="4" t="s">
-        <v>120</v>
       </c>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -5598,7 +5598,7 @@
       </c>
       <c r="K63" s="4"/>
       <c r="L63" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M63" s="4" t="s">
         <v>48</v>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="O63" s="4"/>
       <c r="P63" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q63" s="4">
         <v>1</v>
@@ -5617,7 +5617,7 @@
         <v>50</v>
       </c>
       <c r="S63" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="T63" s="4">
         <v>1</v>
@@ -5647,19 +5647,19 @@
       <c r="AO63" s="6"/>
       <c r="AP63" s="6"/>
     </row>
-    <row r="64" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A64" s="4"/>
       <c r="B64" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F64" s="4" t="s">
         <v>55</v>
@@ -5674,7 +5674,7 @@
       </c>
       <c r="K64" s="4"/>
       <c r="L64" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="M64" s="4" t="s">
         <v>67</v>
@@ -5682,7 +5682,7 @@
       <c r="N64" s="4"/>
       <c r="O64" s="4"/>
       <c r="P64" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q64" s="4">
         <v>1</v>
@@ -5709,10 +5709,10 @@
       <c r="AC64" s="4"/>
       <c r="AD64" s="4"/>
       <c r="AE64" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AF64" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AG64" s="4"/>
       <c r="AH64" s="4"/>
@@ -5725,19 +5725,19 @@
       <c r="AO64" s="6"/>
       <c r="AP64" s="6"/>
     </row>
-    <row r="65" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A65" s="4"/>
       <c r="B65" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F65" s="4" t="s">
         <v>55</v>
@@ -5758,7 +5758,7 @@
       <c r="N65" s="4"/>
       <c r="O65" s="4"/>
       <c r="P65" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q65" s="4">
         <v>30</v>
@@ -5785,10 +5785,10 @@
       <c r="AC65" s="4"/>
       <c r="AD65" s="4"/>
       <c r="AE65" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="AF65" s="4" t="s">
         <v>128</v>
-      </c>
-      <c r="AF65" s="4" t="s">
-        <v>129</v>
       </c>
       <c r="AG65" s="4"/>
       <c r="AH65" s="4"/>

</xml_diff>

<commit_message>
move criteria tables back to inst/extdata
</commit_message>
<xml_diff>
--- a/inst/extdata/blackfeet_tribe_criteria_crosswalk.xlsx
+++ b/inst/extdata/blackfeet_tribe_criteria_crosswalk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kwong01\TADACommunityHub\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB60F2B-4287-4E1F-B327-A1104AEB08CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2059C3BF-FEA9-4515-96A4-28B4B0F0BCB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9CAA114B-CC1B-4AA7-94E1-A6CD4C5CB112}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" xr2:uid="{9CAA114B-CC1B-4AA7-94E1-A6CD4C5CB112}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -134,9 +134,6 @@
     <t>EquationType</t>
   </si>
   <si>
-    <t>Equation</t>
-  </si>
-  <si>
     <t>hardness_param_1</t>
   </si>
   <si>
@@ -498,6 +495,9 @@
   </si>
   <si>
     <t>CFU/100ML</t>
+  </si>
+  <si>
+    <t>EquationFormula</t>
   </si>
 </sst>
 </file>
@@ -907,19 +907,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{057945F5-944B-4C7F-AE65-F75344336C85}">
   <dimension ref="A1:AP65"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.1796875" style="3"/>
+    <col min="1" max="2" width="9.140625" style="3"/>
     <col min="3" max="3" width="27" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.54296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="18" width="9.1796875" style="3"/>
-    <col min="19" max="19" width="19.7265625" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="31" width="9.1796875" style="3"/>
-    <col min="32" max="32" width="12.453125" style="3" customWidth="1"/>
-    <col min="33" max="16384" width="9.1796875" style="3"/>
+    <col min="4" max="4" width="31.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="18" width="9.140625" style="3"/>
+    <col min="19" max="19" width="19.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="31" width="9.140625" style="3"/>
+    <col min="32" max="32" width="12.42578125" style="3" customWidth="1"/>
+    <col min="33" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:42" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1014,88 +1014,88 @@
         <v>30</v>
       </c>
       <c r="AF1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="AG1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
       <c r="B2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
       <c r="M2" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N2" s="4"/>
       <c r="O2" s="4">
         <v>20000</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q2" s="4">
         <v>4</v>
       </c>
       <c r="R2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4">
+        <v>1</v>
+      </c>
+      <c r="U2" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="T2" s="4">
-        <v>1</v>
-      </c>
-      <c r="U2" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="V2" s="4"/>
       <c r="W2" s="4"/>
@@ -1119,57 +1119,57 @@
       <c r="AO2" s="6"/>
       <c r="AP2" s="6"/>
     </row>
-    <row r="3" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K3" s="4"/>
       <c r="L3" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N3" s="4"/>
       <c r="O3" s="4">
         <v>1.5</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q3" s="4">
         <v>30</v>
       </c>
       <c r="R3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S3" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S3" s="4" t="s">
+      <c r="T3" s="4">
+        <v>1</v>
+      </c>
+      <c r="U3" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="T3" s="4">
-        <v>1</v>
-      </c>
-      <c r="U3" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="V3" s="4"/>
       <c r="W3" s="4"/>
@@ -1193,57 +1193,57 @@
       <c r="AO3" s="6"/>
       <c r="AP3" s="6"/>
     </row>
-    <row r="4" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N4" s="4"/>
       <c r="O4" s="4">
         <v>3.1</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q4" s="4">
         <v>30</v>
       </c>
       <c r="R4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S4" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S4" s="4" t="s">
+      <c r="T4" s="4">
+        <v>1</v>
+      </c>
+      <c r="U4" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="T4" s="4">
-        <v>1</v>
-      </c>
-      <c r="U4" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="V4" s="4"/>
       <c r="W4" s="4"/>
@@ -1267,53 +1267,53 @@
       <c r="AO4" s="6"/>
       <c r="AP4" s="6"/>
     </row>
-    <row r="5" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>59</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N5" s="4"/>
       <c r="O5" s="4">
         <v>5.6</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q5" s="4">
         <v>30</v>
       </c>
       <c r="R5" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S5" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S5" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T5" s="4">
         <v>1</v>
       </c>
       <c r="U5" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -1337,53 +1337,53 @@
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
     </row>
-    <row r="6" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>59</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N6" s="4"/>
       <c r="O6" s="4">
         <v>5.6</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q6" s="4">
         <v>30</v>
       </c>
       <c r="R6" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S6" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S6" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T6" s="4">
         <v>1</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -1407,57 +1407,57 @@
       <c r="AO6" s="6"/>
       <c r="AP6" s="6"/>
     </row>
-    <row r="7" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>63</v>
-      </c>
       <c r="F7" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N7" s="4"/>
       <c r="O7" s="4">
         <v>340</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q7" s="4">
         <v>1</v>
       </c>
       <c r="R7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S7" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S7" s="4" t="s">
+      <c r="T7" s="4">
+        <v>1</v>
+      </c>
+      <c r="U7" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="T7" s="4">
-        <v>1</v>
-      </c>
-      <c r="U7" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -1481,55 +1481,55 @@
       <c r="AO7" s="6"/>
       <c r="AP7" s="6"/>
     </row>
-    <row r="8" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>63</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N8" s="4"/>
       <c r="O8" s="4">
         <v>150</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q8" s="4">
         <v>4</v>
       </c>
       <c r="R8" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S8" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S8" s="4" t="s">
+      <c r="T8" s="4">
+        <v>1</v>
+      </c>
+      <c r="U8" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="T8" s="4">
-        <v>1</v>
-      </c>
-      <c r="U8" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
@@ -1553,53 +1553,53 @@
       <c r="AO8" s="6"/>
       <c r="AP8" s="6"/>
     </row>
-    <row r="9" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>63</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N9" s="4"/>
       <c r="O9" s="4">
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q9" s="4">
         <v>30</v>
       </c>
       <c r="R9" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S9" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S9" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T9" s="4">
         <v>1</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
@@ -1623,55 +1623,55 @@
       <c r="AO9" s="6"/>
       <c r="AP9" s="6"/>
     </row>
-    <row r="10" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>66</v>
-      </c>
       <c r="F10" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
       <c r="P10" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q10" s="4">
         <v>1</v>
       </c>
       <c r="R10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T10" s="4">
         <v>1</v>
       </c>
       <c r="U10" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
@@ -1683,10 +1683,10 @@
       <c r="AC10" s="4"/>
       <c r="AD10" s="4"/>
       <c r="AE10" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AF10" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AG10" s="4"/>
       <c r="AH10" s="4"/>
@@ -1699,55 +1699,55 @@
       <c r="AO10" s="6"/>
       <c r="AP10" s="6"/>
     </row>
-    <row r="11" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>66</v>
-      </c>
       <c r="F11" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
       <c r="P11" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q11" s="4">
         <v>30</v>
       </c>
       <c r="R11" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S11" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S11" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T11" s="4">
         <v>1</v>
       </c>
       <c r="U11" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V11" s="4"/>
       <c r="W11" s="4"/>
@@ -1759,10 +1759,10 @@
       <c r="AC11" s="4"/>
       <c r="AD11" s="4"/>
       <c r="AE11" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AF11" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AG11" s="4"/>
       <c r="AH11" s="4"/>
@@ -1775,55 +1775,55 @@
       <c r="AO11" s="6"/>
       <c r="AP11" s="6"/>
     </row>
-    <row r="12" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N12" s="4"/>
       <c r="O12" s="4">
         <v>1300</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q12" s="4">
         <v>1</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T12" s="4">
         <v>1</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V12" s="4"/>
       <c r="W12" s="4"/>
@@ -1847,57 +1847,57 @@
       <c r="AO12" s="6"/>
       <c r="AP12" s="6"/>
     </row>
-    <row r="13" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="F13" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I13" s="4"/>
       <c r="J13" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N13" s="4"/>
       <c r="O13" s="4">
         <v>2.5</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q13" s="4">
         <v>30</v>
       </c>
       <c r="R13" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S13" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S13" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T13" s="4">
         <v>1</v>
       </c>
       <c r="U13" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V13" s="4"/>
       <c r="W13" s="4"/>
@@ -1921,57 +1921,57 @@
       <c r="AO13" s="6"/>
       <c r="AP13" s="6"/>
     </row>
-    <row r="14" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="F14" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I14" s="4"/>
       <c r="J14" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N14" s="4"/>
       <c r="O14" s="4">
         <v>1.4</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q14" s="4">
         <v>1</v>
       </c>
       <c r="R14" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T14" s="4">
         <v>1</v>
       </c>
       <c r="U14" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V14" s="4"/>
       <c r="W14" s="4"/>
@@ -1995,55 +1995,55 @@
       <c r="AO14" s="6"/>
       <c r="AP14" s="6"/>
     </row>
-    <row r="15" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="F15" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N15" s="4"/>
       <c r="O15" s="4">
         <v>0.05</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q15" s="4">
         <v>1</v>
       </c>
       <c r="R15" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T15" s="4">
         <v>1</v>
       </c>
       <c r="U15" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V15" s="4"/>
       <c r="W15" s="4"/>
@@ -2067,55 +2067,55 @@
       <c r="AO15" s="6"/>
       <c r="AP15" s="6"/>
     </row>
-    <row r="16" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
       <c r="B16" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="F16" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N16" s="4"/>
       <c r="O16" s="4">
         <v>5.0999999999999997E-2</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q16" s="4">
         <v>30</v>
       </c>
       <c r="R16" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S16" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S16" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T16" s="4">
         <v>1</v>
       </c>
       <c r="U16" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V16" s="4"/>
       <c r="W16" s="4"/>
@@ -2139,53 +2139,53 @@
       <c r="AO16" s="6"/>
       <c r="AP16" s="6"/>
     </row>
-    <row r="17" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
       <c r="M17" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N17" s="4"/>
       <c r="O17" s="4">
         <v>0.3</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q17" s="4">
         <v>30</v>
       </c>
       <c r="R17" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S17" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T17" s="4">
         <v>1</v>
       </c>
       <c r="U17" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V17" s="4"/>
       <c r="W17" s="4"/>
@@ -2209,53 +2209,53 @@
       <c r="AO17" s="6"/>
       <c r="AP17" s="6"/>
     </row>
-    <row r="18" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K18" s="4"/>
       <c r="L18" s="4"/>
       <c r="M18" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N18" s="4"/>
       <c r="O18" s="4">
         <v>0.3</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q18" s="4">
         <v>30</v>
       </c>
       <c r="R18" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S18" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S18" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T18" s="4">
         <v>1</v>
       </c>
       <c r="U18" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V18" s="4"/>
       <c r="W18" s="4"/>
@@ -2279,57 +2279,57 @@
       <c r="AO18" s="6"/>
       <c r="AP18" s="6"/>
     </row>
-    <row r="19" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I19" s="4"/>
       <c r="J19" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
       <c r="M19" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N19" s="4"/>
       <c r="O19" s="4">
         <v>16</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q19" s="4">
         <v>1</v>
       </c>
       <c r="R19" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T19" s="4">
         <v>1</v>
       </c>
       <c r="U19" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V19" s="4"/>
       <c r="W19" s="4"/>
@@ -2353,57 +2353,57 @@
       <c r="AO19" s="6"/>
       <c r="AP19" s="6"/>
     </row>
-    <row r="20" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I20" s="4"/>
       <c r="J20" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K20" s="4"/>
       <c r="L20" s="4"/>
       <c r="M20" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N20" s="4"/>
       <c r="O20" s="4">
         <v>11</v>
       </c>
       <c r="P20" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q20" s="4">
         <v>30</v>
       </c>
       <c r="R20" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S20" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S20" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T20" s="4">
         <v>1</v>
       </c>
       <c r="U20" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V20" s="4"/>
       <c r="W20" s="4"/>
@@ -2427,55 +2427,55 @@
       <c r="AO20" s="6"/>
       <c r="AP20" s="6"/>
     </row>
-    <row r="21" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>83</v>
-      </c>
       <c r="F21" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K21" s="4"/>
       <c r="L21" s="4"/>
       <c r="M21" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N21" s="4"/>
       <c r="O21" s="4">
         <v>610</v>
       </c>
       <c r="P21" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q21" s="4">
         <v>1</v>
       </c>
       <c r="R21" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T21" s="4">
         <v>1</v>
       </c>
       <c r="U21" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V21" s="4"/>
       <c r="W21" s="4"/>
@@ -2499,55 +2499,55 @@
       <c r="AO21" s="6"/>
       <c r="AP21" s="6"/>
     </row>
-    <row r="22" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
       <c r="B22" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>83</v>
-      </c>
       <c r="F22" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K22" s="4"/>
       <c r="L22" s="4"/>
       <c r="M22" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N22" s="4"/>
       <c r="O22" s="4">
         <v>4600</v>
       </c>
       <c r="P22" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q22" s="4">
         <v>30</v>
       </c>
       <c r="R22" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S22" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S22" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T22" s="4">
         <v>1</v>
       </c>
       <c r="U22" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V22" s="4"/>
       <c r="W22" s="4"/>
@@ -2571,55 +2571,55 @@
       <c r="AO22" s="6"/>
       <c r="AP22" s="6"/>
     </row>
-    <row r="23" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
       <c r="B23" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>54</v>
-      </c>
       <c r="F23" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
       <c r="M23" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N23" s="4"/>
       <c r="O23" s="4">
         <v>170</v>
       </c>
       <c r="P23" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q23" s="4">
         <v>1</v>
       </c>
       <c r="R23" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T23" s="4">
         <v>1</v>
       </c>
       <c r="U23" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V23" s="4"/>
       <c r="W23" s="4"/>
@@ -2643,55 +2643,55 @@
       <c r="AO23" s="6"/>
       <c r="AP23" s="6"/>
     </row>
-    <row r="24" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
       <c r="B24" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>54</v>
-      </c>
       <c r="F24" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
       <c r="J24" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
       <c r="M24" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N24" s="4"/>
       <c r="O24" s="4">
         <v>4200</v>
       </c>
       <c r="P24" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q24" s="4">
         <v>30</v>
       </c>
       <c r="R24" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S24" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S24" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T24" s="4">
         <v>1</v>
       </c>
       <c r="U24" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V24" s="4"/>
       <c r="W24" s="4"/>
@@ -2715,55 +2715,55 @@
       <c r="AO24" s="6"/>
       <c r="AP24" s="6"/>
     </row>
-    <row r="25" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D25" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>85</v>
-      </c>
       <c r="F25" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
       <c r="J25" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K25" s="4"/>
       <c r="L25" s="4"/>
       <c r="M25" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N25" s="4"/>
       <c r="O25" s="4">
         <v>0.24</v>
       </c>
       <c r="P25" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q25" s="4">
         <v>1</v>
       </c>
       <c r="R25" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S25" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T25" s="4">
         <v>1</v>
       </c>
       <c r="U25" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V25" s="4"/>
       <c r="W25" s="4"/>
@@ -2787,55 +2787,55 @@
       <c r="AO25" s="6"/>
       <c r="AP25" s="6"/>
     </row>
-    <row r="26" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C26" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>85</v>
-      </c>
       <c r="F26" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
       <c r="J26" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K26" s="4"/>
       <c r="L26" s="4"/>
       <c r="M26" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N26" s="4"/>
       <c r="O26" s="4">
         <v>0.47</v>
       </c>
       <c r="P26" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q26" s="4">
         <v>30</v>
       </c>
       <c r="R26" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S26" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S26" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T26" s="4">
         <v>1</v>
       </c>
       <c r="U26" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V26" s="4"/>
       <c r="W26" s="4"/>
@@ -2859,55 +2859,55 @@
       <c r="AO26" s="6"/>
       <c r="AP26" s="6"/>
     </row>
-    <row r="27" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C27" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D27" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>87</v>
-      </c>
       <c r="F27" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K27" s="4"/>
       <c r="L27" s="4"/>
       <c r="M27" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N27" s="4"/>
       <c r="O27" s="4">
         <v>7400</v>
       </c>
       <c r="P27" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q27" s="4">
         <v>1</v>
       </c>
       <c r="R27" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S27" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T27" s="4">
         <v>1</v>
       </c>
       <c r="U27" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V27" s="4"/>
       <c r="W27" s="4"/>
@@ -2931,55 +2931,55 @@
       <c r="AO27" s="6"/>
       <c r="AP27" s="6"/>
     </row>
-    <row r="28" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>87</v>
-      </c>
       <c r="F28" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K28" s="4"/>
       <c r="L28" s="4"/>
       <c r="M28" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N28" s="4"/>
       <c r="O28" s="4">
         <v>26000</v>
       </c>
       <c r="P28" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q28" s="4">
         <v>30</v>
       </c>
       <c r="R28" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S28" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S28" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T28" s="4">
         <v>1</v>
       </c>
       <c r="U28" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V28" s="4"/>
       <c r="W28" s="4"/>
@@ -3003,55 +3003,55 @@
       <c r="AO28" s="6"/>
       <c r="AP28" s="6"/>
     </row>
-    <row r="29" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C29" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I29" s="4"/>
       <c r="J29" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
       <c r="M29" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N29" s="4"/>
       <c r="O29" s="4">
         <v>22</v>
       </c>
       <c r="P29" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q29" s="4">
         <v>1</v>
       </c>
       <c r="R29" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S29" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T29" s="4">
         <v>1</v>
       </c>
       <c r="U29" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V29" s="4"/>
       <c r="W29" s="4"/>
@@ -3075,55 +3075,55 @@
       <c r="AO29" s="6"/>
       <c r="AP29" s="6"/>
     </row>
-    <row r="30" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
       <c r="B30" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C30" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I30" s="4"/>
       <c r="J30" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K30" s="4"/>
       <c r="L30" s="4"/>
       <c r="M30" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N30" s="4"/>
       <c r="O30" s="4">
         <v>5.2</v>
       </c>
       <c r="P30" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q30" s="4">
         <v>30</v>
       </c>
       <c r="R30" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S30" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S30" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T30" s="4">
         <v>1</v>
       </c>
       <c r="U30" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V30" s="4"/>
       <c r="W30" s="4"/>
@@ -3147,53 +3147,53 @@
       <c r="AO30" s="6"/>
       <c r="AP30" s="6"/>
     </row>
-    <row r="31" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
       <c r="B31" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C31" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
       <c r="J31" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K31" s="4"/>
       <c r="L31" s="4"/>
       <c r="M31" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N31" s="4"/>
       <c r="O31" s="4">
         <v>4</v>
       </c>
       <c r="P31" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q31" s="4">
         <v>1</v>
       </c>
       <c r="R31" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S31" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T31" s="4">
         <v>1</v>
       </c>
       <c r="U31" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="4"/>
@@ -3217,53 +3217,53 @@
       <c r="AO31" s="6"/>
       <c r="AP31" s="6"/>
     </row>
-    <row r="32" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
       <c r="B32" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C32" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
       <c r="J32" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K32" s="4"/>
       <c r="L32" s="4"/>
       <c r="M32" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N32" s="4"/>
       <c r="O32" s="4">
         <v>400</v>
       </c>
       <c r="P32" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q32" s="4">
         <v>30</v>
       </c>
       <c r="R32" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S32" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S32" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T32" s="4">
         <v>1</v>
       </c>
       <c r="U32" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V32" s="4"/>
       <c r="W32" s="4"/>
@@ -3287,53 +3287,53 @@
       <c r="AO32" s="6"/>
       <c r="AP32" s="6"/>
     </row>
-    <row r="33" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C33" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E33" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>91</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
       <c r="J33" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K33" s="4"/>
       <c r="L33" s="4"/>
       <c r="M33" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N33" s="4"/>
       <c r="O33" s="4">
         <v>7000000</v>
       </c>
       <c r="P33" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="Q33" s="4">
         <v>1</v>
       </c>
       <c r="R33" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S33" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T33" s="4">
         <v>1</v>
       </c>
       <c r="U33" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V33" s="4"/>
       <c r="W33" s="4"/>
@@ -3357,55 +3357,55 @@
       <c r="AO33" s="6"/>
       <c r="AP33" s="6"/>
     </row>
-    <row r="34" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
       <c r="B34" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C34" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E34" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D34" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>94</v>
-      </c>
       <c r="F34" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I34" s="4"/>
       <c r="J34" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
       <c r="M34" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N34" s="4"/>
       <c r="O34" s="4"/>
       <c r="P34" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q34" s="4">
         <v>1</v>
       </c>
       <c r="R34" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S34" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T34" s="4">
         <v>1</v>
       </c>
       <c r="U34" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V34" s="4"/>
       <c r="W34" s="4"/>
@@ -3417,10 +3417,10 @@
       <c r="AC34" s="4"/>
       <c r="AD34" s="4"/>
       <c r="AE34" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF34" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AG34" s="4">
         <v>1.1366719999999999</v>
@@ -3443,55 +3443,55 @@
       <c r="AO34" s="6"/>
       <c r="AP34" s="6"/>
     </row>
-    <row r="35" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C35" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D35" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>94</v>
-      </c>
       <c r="F35" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I35" s="4"/>
       <c r="J35" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
       <c r="M35" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N35" s="4"/>
       <c r="O35" s="4"/>
       <c r="P35" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q35" s="4">
         <v>30</v>
       </c>
       <c r="R35" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S35" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S35" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T35" s="4">
         <v>1</v>
       </c>
       <c r="U35" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V35" s="4"/>
       <c r="W35" s="4"/>
@@ -3503,10 +3503,10 @@
       <c r="AC35" s="4"/>
       <c r="AD35" s="4"/>
       <c r="AE35" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF35" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AG35" s="4">
         <v>1.101672</v>
@@ -3529,55 +3529,55 @@
       <c r="AO35" s="6"/>
       <c r="AP35" s="6"/>
     </row>
-    <row r="36" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
       <c r="B36" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I36" s="4"/>
       <c r="J36" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K36" s="4"/>
       <c r="L36" s="4"/>
       <c r="M36" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N36" s="4"/>
       <c r="O36" s="4"/>
       <c r="P36" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q36" s="4">
         <v>1</v>
       </c>
       <c r="R36" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S36" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T36" s="4">
         <v>1</v>
       </c>
       <c r="U36" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V36" s="4"/>
       <c r="W36" s="4"/>
@@ -3589,10 +3589,10 @@
       <c r="AC36" s="4"/>
       <c r="AD36" s="4"/>
       <c r="AE36" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF36" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AG36" s="4"/>
       <c r="AH36" s="4"/>
@@ -3611,55 +3611,55 @@
       <c r="AO36" s="6"/>
       <c r="AP36" s="6"/>
     </row>
-    <row r="37" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I37" s="4"/>
       <c r="J37" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K37" s="4"/>
       <c r="L37" s="4"/>
       <c r="M37" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N37" s="4"/>
       <c r="O37" s="4"/>
       <c r="P37" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q37" s="4">
         <v>30</v>
       </c>
       <c r="R37" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S37" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S37" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T37" s="4">
         <v>1</v>
       </c>
       <c r="U37" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V37" s="4"/>
       <c r="W37" s="4"/>
@@ -3671,10 +3671,10 @@
       <c r="AC37" s="4"/>
       <c r="AD37" s="4"/>
       <c r="AE37" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF37" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AG37" s="4"/>
       <c r="AH37" s="4"/>
@@ -3693,55 +3693,55 @@
       <c r="AO37" s="6"/>
       <c r="AP37" s="6"/>
     </row>
-    <row r="38" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
       <c r="B38" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C38" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D38" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="F38" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I38" s="4"/>
       <c r="J38" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K38" s="4"/>
       <c r="L38" s="4"/>
       <c r="M38" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N38" s="4"/>
       <c r="O38" s="4"/>
       <c r="P38" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q38" s="4">
         <v>1</v>
       </c>
       <c r="R38" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S38" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T38" s="4">
         <v>1</v>
       </c>
       <c r="U38" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V38" s="4"/>
       <c r="W38" s="4"/>
@@ -3753,10 +3753,10 @@
       <c r="AC38" s="4"/>
       <c r="AD38" s="4"/>
       <c r="AE38" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF38" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AG38" s="4">
         <v>1.4620299999999999</v>
@@ -3779,55 +3779,55 @@
       <c r="AO38" s="6"/>
       <c r="AP38" s="6"/>
     </row>
-    <row r="39" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C39" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D39" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="F39" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N39" s="4"/>
       <c r="O39" s="4"/>
       <c r="P39" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q39" s="4">
         <v>30</v>
       </c>
       <c r="R39" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S39" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S39" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T39" s="4">
         <v>1</v>
       </c>
       <c r="U39" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V39" s="4"/>
       <c r="W39" s="4"/>
@@ -3839,10 +3839,10 @@
       <c r="AC39" s="4"/>
       <c r="AD39" s="4"/>
       <c r="AE39" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF39" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AG39" s="4">
         <v>1.4620299999999999</v>
@@ -3865,55 +3865,55 @@
       <c r="AO39" s="6"/>
       <c r="AP39" s="6"/>
     </row>
-    <row r="40" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C40" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E40" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D40" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>83</v>
-      </c>
       <c r="F40" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N40" s="4"/>
       <c r="O40" s="4"/>
       <c r="P40" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q40" s="4">
         <v>1</v>
       </c>
       <c r="R40" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S40" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T40" s="4">
         <v>1</v>
       </c>
       <c r="U40" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V40" s="4"/>
       <c r="W40" s="4"/>
@@ -3925,10 +3925,10 @@
       <c r="AC40" s="4"/>
       <c r="AD40" s="4"/>
       <c r="AE40" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF40" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AG40" s="4"/>
       <c r="AH40" s="4"/>
@@ -3947,55 +3947,55 @@
       <c r="AO40" s="6"/>
       <c r="AP40" s="6"/>
     </row>
-    <row r="41" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>83</v>
-      </c>
       <c r="F41" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G41" s="4"/>
       <c r="H41" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
       <c r="M41" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N41" s="4"/>
       <c r="O41" s="4"/>
       <c r="P41" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q41" s="4">
         <v>30</v>
       </c>
       <c r="R41" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S41" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S41" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T41" s="4">
         <v>1</v>
       </c>
       <c r="U41" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V41" s="4"/>
       <c r="W41" s="4"/>
@@ -4007,10 +4007,10 @@
       <c r="AC41" s="4"/>
       <c r="AD41" s="4"/>
       <c r="AE41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF41" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AG41" s="4"/>
       <c r="AH41" s="4"/>
@@ -4029,55 +4029,55 @@
       <c r="AO41" s="6"/>
       <c r="AP41" s="6"/>
     </row>
-    <row r="42" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
       <c r="B42" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C42" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E42" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D42" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>98</v>
-      </c>
       <c r="F42" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K42" s="4"/>
       <c r="L42" s="4"/>
       <c r="M42" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N42" s="4"/>
       <c r="O42" s="4"/>
       <c r="P42" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q42" s="4">
         <v>1</v>
       </c>
       <c r="R42" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S42" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T42" s="4">
         <v>1</v>
       </c>
       <c r="U42" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V42" s="4"/>
       <c r="W42" s="4"/>
@@ -4089,10 +4089,10 @@
       <c r="AC42" s="4"/>
       <c r="AD42" s="4"/>
       <c r="AE42" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF42" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AG42" s="4"/>
       <c r="AH42" s="4"/>
@@ -4111,55 +4111,55 @@
       <c r="AO42" s="6"/>
       <c r="AP42" s="6"/>
     </row>
-    <row r="43" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="4"/>
       <c r="B43" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C43" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D43" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>87</v>
-      </c>
       <c r="F43" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I43" s="4"/>
       <c r="J43" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K43" s="4"/>
       <c r="L43" s="4"/>
       <c r="M43" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N43" s="4"/>
       <c r="O43" s="4"/>
       <c r="P43" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q43" s="4">
         <v>1</v>
       </c>
       <c r="R43" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S43" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T43" s="4">
         <v>1</v>
       </c>
       <c r="U43" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V43" s="4"/>
       <c r="W43" s="4"/>
@@ -4171,10 +4171,10 @@
       <c r="AC43" s="4"/>
       <c r="AD43" s="4"/>
       <c r="AE43" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF43" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AG43" s="4"/>
       <c r="AH43" s="4"/>
@@ -4193,55 +4193,55 @@
       <c r="AO43" s="6"/>
       <c r="AP43" s="6"/>
     </row>
-    <row r="44" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="4"/>
       <c r="B44" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C44" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D44" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>87</v>
-      </c>
       <c r="F44" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G44" s="4"/>
       <c r="H44" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I44" s="4"/>
       <c r="J44" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K44" s="4"/>
       <c r="L44" s="4"/>
       <c r="M44" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N44" s="4"/>
       <c r="O44" s="4"/>
       <c r="P44" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q44" s="4">
         <v>30</v>
       </c>
       <c r="R44" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S44" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S44" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T44" s="4">
         <v>1</v>
       </c>
       <c r="U44" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V44" s="4"/>
       <c r="W44" s="4"/>
@@ -4253,10 +4253,10 @@
       <c r="AC44" s="4"/>
       <c r="AD44" s="4"/>
       <c r="AE44" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AF44" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AG44" s="4"/>
       <c r="AH44" s="4"/>
@@ -4275,53 +4275,53 @@
       <c r="AO44" s="6"/>
       <c r="AP44" s="6"/>
     </row>
-    <row r="45" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="4"/>
       <c r="B45" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C45" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>100</v>
       </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
       <c r="J45" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K45" s="4"/>
       <c r="L45" s="4"/>
       <c r="M45" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N45" s="4"/>
       <c r="O45" s="4">
         <v>1000</v>
       </c>
       <c r="P45" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q45" s="4">
         <v>1</v>
       </c>
       <c r="R45" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S45" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T45" s="4">
         <v>1</v>
       </c>
       <c r="U45" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V45" s="4"/>
       <c r="W45" s="4"/>
@@ -4345,55 +4345,55 @@
       <c r="AO45" s="6"/>
       <c r="AP45" s="6"/>
     </row>
-    <row r="46" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="4"/>
       <c r="B46" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C46" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E46" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>102</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I46" s="4"/>
       <c r="J46" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K46" s="4"/>
       <c r="L46" s="4"/>
       <c r="M46" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N46" s="4"/>
       <c r="O46" s="4">
         <v>860000</v>
       </c>
       <c r="P46" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q46" s="4">
         <v>1</v>
       </c>
       <c r="R46" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S46" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T46" s="4">
         <v>1</v>
       </c>
       <c r="U46" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V46" s="4"/>
       <c r="W46" s="4"/>
@@ -4417,55 +4417,55 @@
       <c r="AO46" s="6"/>
       <c r="AP46" s="6"/>
     </row>
-    <row r="47" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="4"/>
       <c r="B47" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C47" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E47" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>102</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I47" s="4"/>
       <c r="J47" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K47" s="4"/>
       <c r="L47" s="4"/>
       <c r="M47" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N47" s="4"/>
       <c r="O47" s="4">
         <v>230000</v>
       </c>
       <c r="P47" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q47" s="4">
         <v>30</v>
       </c>
       <c r="R47" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S47" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S47" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T47" s="4">
         <v>1</v>
       </c>
       <c r="U47" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V47" s="4"/>
       <c r="W47" s="4"/>
@@ -4489,57 +4489,57 @@
       <c r="AO47" s="6"/>
       <c r="AP47" s="6"/>
     </row>
-    <row r="48" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="4"/>
       <c r="B48" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C48" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E48" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D48" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>104</v>
-      </c>
       <c r="F48" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G48" s="4"/>
       <c r="H48" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I48" s="4"/>
       <c r="J48" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="4"/>
       <c r="M48" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N48" s="4"/>
       <c r="O48" s="4">
         <v>19</v>
       </c>
       <c r="P48" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q48" s="4">
         <v>1</v>
       </c>
       <c r="R48" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S48" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T48" s="4">
         <v>1</v>
       </c>
       <c r="U48" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V48" s="4"/>
       <c r="W48" s="4"/>
@@ -4563,57 +4563,57 @@
       <c r="AO48" s="6"/>
       <c r="AP48" s="6"/>
     </row>
-    <row r="49" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
       <c r="B49" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C49" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E49" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>104</v>
-      </c>
       <c r="F49" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G49" s="4"/>
       <c r="H49" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I49" s="4"/>
       <c r="J49" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K49" s="4"/>
       <c r="L49" s="4"/>
       <c r="M49" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N49" s="4"/>
       <c r="O49" s="4">
         <v>11</v>
       </c>
       <c r="P49" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q49" s="4">
         <v>30</v>
       </c>
       <c r="R49" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S49" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S49" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T49" s="4">
         <v>1</v>
       </c>
       <c r="U49" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V49" s="4"/>
       <c r="W49" s="4"/>
@@ -4637,55 +4637,55 @@
       <c r="AO49" s="6"/>
       <c r="AP49" s="6"/>
     </row>
-    <row r="50" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="4"/>
       <c r="B50" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C50" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E50" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>106</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I50" s="4"/>
       <c r="J50" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K50" s="4"/>
       <c r="L50" s="4"/>
       <c r="M50" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N50" s="4"/>
       <c r="O50" s="4">
         <v>1000</v>
       </c>
       <c r="P50" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q50" s="4">
         <v>30</v>
       </c>
       <c r="R50" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S50" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S50" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T50" s="4">
         <v>1</v>
       </c>
       <c r="U50" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V50" s="4"/>
       <c r="W50" s="4"/>
@@ -4709,53 +4709,53 @@
       <c r="AO50" s="6"/>
       <c r="AP50" s="6"/>
     </row>
-    <row r="51" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="4"/>
       <c r="B51" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
       <c r="J51" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K51" s="4"/>
       <c r="L51" s="4"/>
       <c r="M51" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N51" s="4"/>
       <c r="O51" s="4">
         <v>10000</v>
       </c>
       <c r="P51" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q51" s="4">
         <v>1</v>
       </c>
       <c r="R51" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S51" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T51" s="4">
         <v>1</v>
       </c>
       <c r="U51" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V51" s="4"/>
       <c r="W51" s="4"/>
@@ -4779,33 +4779,33 @@
       <c r="AO51" s="6"/>
       <c r="AP51" s="6"/>
     </row>
-    <row r="52" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="4"/>
       <c r="B52" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C52" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E52" s="4" t="s">
         <v>108</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E52" s="4" t="s">
-        <v>109</v>
       </c>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I52" s="4"/>
       <c r="J52" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K52" s="4"/>
       <c r="L52" s="4"/>
       <c r="M52" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N52" s="4">
         <v>6.5</v>
@@ -4814,22 +4814,22 @@
         <v>9</v>
       </c>
       <c r="P52" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Q52" s="4">
         <v>7</v>
       </c>
       <c r="R52" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S52" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T52" s="4">
         <v>1</v>
       </c>
       <c r="U52" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V52" s="4"/>
       <c r="W52" s="4"/>
@@ -4853,31 +4853,31 @@
       <c r="AO52" s="6"/>
       <c r="AP52" s="6"/>
     </row>
-    <row r="53" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
       <c r="B53" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C53" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E53" s="4" t="s">
         <v>108</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>109</v>
       </c>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
       <c r="J53" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K53" s="4"/>
       <c r="L53" s="4"/>
       <c r="M53" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N53" s="4">
         <v>5</v>
@@ -4886,22 +4886,22 @@
         <v>9</v>
       </c>
       <c r="P53" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q53" s="4">
+        <v>1</v>
+      </c>
+      <c r="R53" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S53" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="Q53" s="4">
-        <v>1</v>
-      </c>
-      <c r="R53" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="S53" s="4" t="s">
-        <v>111</v>
-      </c>
       <c r="T53" s="4">
         <v>1</v>
       </c>
       <c r="U53" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V53" s="4"/>
       <c r="W53" s="4"/>
@@ -4925,55 +4925,55 @@
       <c r="AO53" s="6"/>
       <c r="AP53" s="6"/>
     </row>
-    <row r="54" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="4"/>
       <c r="B54" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
       <c r="J54" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K54" s="4"/>
       <c r="L54" s="4"/>
       <c r="M54" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N54" s="4"/>
       <c r="O54" s="4">
         <v>250000</v>
       </c>
       <c r="P54" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q54" s="4">
         <v>1</v>
       </c>
       <c r="R54" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S54" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T54" s="4">
         <v>1</v>
       </c>
       <c r="U54" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V54" s="4"/>
       <c r="W54" s="4"/>
@@ -4997,53 +4997,53 @@
       <c r="AO54" s="6"/>
       <c r="AP54" s="6"/>
     </row>
-    <row r="55" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="4"/>
       <c r="B55" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4"/>
       <c r="J55" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K55" s="4"/>
       <c r="L55" s="4"/>
       <c r="M55" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N55" s="4"/>
       <c r="O55" s="4">
         <v>126</v>
       </c>
       <c r="P55" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Q55" s="4">
         <v>90</v>
       </c>
       <c r="R55" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S55" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="T55" s="4">
         <v>1</v>
       </c>
       <c r="U55" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V55" s="4"/>
       <c r="W55" s="4"/>
@@ -5067,53 +5067,53 @@
       <c r="AO55" s="6"/>
       <c r="AP55" s="6"/>
     </row>
-    <row r="56" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="4"/>
       <c r="B56" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
       <c r="J56" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K56" s="4"/>
       <c r="L56" s="4"/>
       <c r="M56" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N56" s="4"/>
       <c r="O56" s="4">
         <v>410</v>
       </c>
       <c r="P56" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Q56" s="4">
         <v>90</v>
       </c>
       <c r="R56" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S56" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="S56" s="4" t="s">
-        <v>51</v>
       </c>
       <c r="T56" s="4">
         <v>10</v>
       </c>
       <c r="U56" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="V56" s="4"/>
       <c r="W56" s="4"/>
@@ -5137,53 +5137,53 @@
       <c r="AO56" s="6"/>
       <c r="AP56" s="6"/>
     </row>
-    <row r="57" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="4"/>
       <c r="B57" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
       <c r="I57" s="4"/>
       <c r="J57" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K57" s="4"/>
       <c r="L57" s="4"/>
       <c r="M57" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N57" s="4"/>
       <c r="O57" s="4">
         <v>8</v>
       </c>
       <c r="P57" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q57" s="4">
         <v>1</v>
       </c>
       <c r="R57" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S57" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T57" s="4">
         <v>1</v>
       </c>
       <c r="U57" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="V57" s="4"/>
       <c r="W57" s="4"/>
@@ -5207,53 +5207,53 @@
       <c r="AO57" s="6"/>
       <c r="AP57" s="6"/>
     </row>
-    <row r="58" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="4"/>
       <c r="B58" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
       <c r="I58" s="4"/>
       <c r="J58" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K58" s="4"/>
       <c r="L58" s="4"/>
       <c r="M58" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N58" s="4"/>
       <c r="O58" s="4">
         <v>15</v>
       </c>
       <c r="P58" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q58" s="4">
         <v>1</v>
       </c>
       <c r="R58" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S58" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T58" s="4">
         <v>1</v>
       </c>
       <c r="U58" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="V58" s="4"/>
       <c r="W58" s="4"/>
@@ -5277,57 +5277,57 @@
       <c r="AO58" s="6"/>
       <c r="AP58" s="6"/>
     </row>
-    <row r="59" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="4"/>
       <c r="B59" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E59" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F59" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="F59" s="4" t="s">
-        <v>119</v>
       </c>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
       <c r="I59" s="4"/>
       <c r="J59" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K59" s="4"/>
       <c r="L59" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M59" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N59" s="4">
         <v>9.5</v>
       </c>
       <c r="O59" s="4"/>
       <c r="P59" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q59" s="4">
         <v>7</v>
       </c>
       <c r="R59" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S59" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S59" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T59" s="4">
         <v>1</v>
       </c>
       <c r="U59" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V59" s="4"/>
       <c r="W59" s="4"/>
@@ -5351,57 +5351,57 @@
       <c r="AO59" s="6"/>
       <c r="AP59" s="6"/>
     </row>
-    <row r="60" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="4"/>
       <c r="B60" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E60" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F60" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="F60" s="4" t="s">
-        <v>119</v>
       </c>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
       <c r="I60" s="4"/>
       <c r="J60" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K60" s="4"/>
       <c r="L60" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M60" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N60" s="4">
         <v>6.5</v>
       </c>
       <c r="O60" s="4"/>
       <c r="P60" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q60" s="4">
         <v>30</v>
       </c>
       <c r="R60" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S60" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S60" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="T60" s="4">
         <v>1</v>
       </c>
       <c r="U60" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V60" s="4"/>
       <c r="W60" s="4"/>
@@ -5425,57 +5425,57 @@
       <c r="AO60" s="6"/>
       <c r="AP60" s="6"/>
     </row>
-    <row r="61" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="4"/>
       <c r="B61" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E61" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F61" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="F61" s="4" t="s">
-        <v>119</v>
       </c>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
       <c r="J61" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K61" s="4"/>
       <c r="L61" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M61" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N61" s="4">
         <v>5</v>
       </c>
       <c r="O61" s="4"/>
       <c r="P61" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q61" s="4">
         <v>7</v>
       </c>
       <c r="R61" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S61" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="T61" s="4">
         <v>1</v>
       </c>
       <c r="U61" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V61" s="4"/>
       <c r="W61" s="4"/>
@@ -5499,57 +5499,57 @@
       <c r="AO61" s="6"/>
       <c r="AP61" s="6"/>
     </row>
-    <row r="62" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="4"/>
       <c r="B62" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E62" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F62" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="F62" s="4" t="s">
-        <v>119</v>
       </c>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
       <c r="J62" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K62" s="4"/>
       <c r="L62" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M62" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N62" s="4">
         <v>8</v>
       </c>
       <c r="O62" s="4"/>
       <c r="P62" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q62" s="4">
         <v>1</v>
       </c>
       <c r="R62" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S62" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="T62" s="4">
         <v>1</v>
       </c>
       <c r="U62" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V62" s="4"/>
       <c r="W62" s="4"/>
@@ -5573,57 +5573,57 @@
       <c r="AO62" s="6"/>
       <c r="AP62" s="6"/>
     </row>
-    <row r="63" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="4"/>
       <c r="B63" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E63" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F63" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="F63" s="4" t="s">
-        <v>119</v>
       </c>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
       <c r="I63" s="4"/>
       <c r="J63" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K63" s="4"/>
       <c r="L63" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M63" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N63" s="4">
         <v>4</v>
       </c>
       <c r="O63" s="4"/>
       <c r="P63" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q63" s="4">
         <v>1</v>
       </c>
       <c r="R63" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S63" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="T63" s="4">
         <v>1</v>
       </c>
       <c r="U63" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V63" s="4"/>
       <c r="W63" s="4"/>
@@ -5647,57 +5647,57 @@
       <c r="AO63" s="6"/>
       <c r="AP63" s="6"/>
     </row>
-    <row r="64" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="4"/>
       <c r="B64" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C64" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E64" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D64" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E64" s="4" t="s">
-        <v>126</v>
-      </c>
       <c r="F64" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G64" s="4"/>
       <c r="H64" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I64" s="4"/>
       <c r="J64" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K64" s="4"/>
       <c r="L64" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="M64" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N64" s="4"/>
       <c r="O64" s="4"/>
       <c r="P64" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q64" s="4">
         <v>1</v>
       </c>
       <c r="R64" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S64" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T64" s="4">
         <v>1</v>
       </c>
       <c r="U64" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="V64" s="4"/>
       <c r="W64" s="4"/>
@@ -5709,10 +5709,10 @@
       <c r="AC64" s="4"/>
       <c r="AD64" s="4"/>
       <c r="AE64" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AF64" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AG64" s="4"/>
       <c r="AH64" s="4"/>
@@ -5725,55 +5725,55 @@
       <c r="AO64" s="6"/>
       <c r="AP64" s="6"/>
     </row>
-    <row r="65" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
       <c r="B65" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C65" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E65" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D65" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E65" s="4" t="s">
-        <v>126</v>
-      </c>
       <c r="F65" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G65" s="4"/>
       <c r="H65" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I65" s="4"/>
       <c r="J65" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K65" s="4"/>
       <c r="L65" s="6"/>
       <c r="M65" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N65" s="4"/>
       <c r="O65" s="4"/>
       <c r="P65" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q65" s="4">
         <v>30</v>
       </c>
       <c r="R65" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S65" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S65" s="4" t="s">
+      <c r="T65" s="4">
+        <v>1</v>
+      </c>
+      <c r="U65" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="T65" s="4">
-        <v>1</v>
-      </c>
-      <c r="U65" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="V65" s="4"/>
       <c r="W65" s="4"/>
@@ -5785,10 +5785,10 @@
       <c r="AC65" s="4"/>
       <c r="AD65" s="4"/>
       <c r="AE65" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="AF65" s="4" t="s">
         <v>127</v>
-      </c>
-      <c r="AF65" s="4" t="s">
-        <v>128</v>
       </c>
       <c r="AG65" s="4"/>
       <c r="AH65" s="4"/>

</xml_diff>